<commit_message>
Turn deliveries into a business with staff and tool upgrades
Shipped orders now become delivery jobs with a promised time. Vans earn
credits per drop (early tip, late half pay, rating multiplier) and cost
a little per trip; jobs queue at the depot when the fleet is busy. A new
Vans tab shows the queue, vans on the road, recent drops and seven
upgrades: drivers, training, dispatcher, scanners, route planner, bigger
vans and electric vans. Vans can be selected and inspected.

Also fixes vans driving through each other at the yard gate, keeps
deliveries to shops near the site you run, renames the page title and
eases Eastport's truck rate. Adds two achievements and delivery sheets
to the rules spreadsheet.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014B4MfCeMGRMcDjRmBPkjgy
</commit_message>
<xml_diff>
--- a/WareTrack_game_rules.xlsx
+++ b/WareTrack_game_rules.xlsx
@@ -15,6 +15,8 @@
     <sheet name="Actions" sheetId="5" state="visible" r:id="rId7"/>
     <sheet name="Upgrades" sheetId="6" state="visible" r:id="rId8"/>
     <sheet name="World and traffic" sheetId="7" state="visible" r:id="rId9"/>
+    <sheet name="Deliveries" sheetId="8" state="visible" r:id="rId10"/>
+    <sheet name="Delivery upgrades" sheetId="9" state="visible" r:id="rId11"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -48,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="227" uniqueCount="215">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="256">
   <si>
     <t xml:space="preserve">Shift calculator</t>
   </si>
@@ -693,6 +695,129 @@
   </si>
   <si>
     <t xml:space="preserve">Zooms out to all five sites with a name pin over each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery vans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every shipped order becomes a delivery to a shop. Credits go straight to your balance, in shifts and in free play.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">How it works</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promised time</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Minutes from shipping until the drop is due: 25 + 3 per block of route (+5 with a Dispatcher)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base fee (credits)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">2 + 0.25 per block, then the route-planner and rating multipliers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Early drop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10 or more minutes before the promised time: +25% tip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Late drop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">After the promised time: half pay, and your rating drops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating multiplier</t>
+  </si>
+  <si>
+    <t xml:space="preserve">0.8 + 0.1 × rating (rating 0–5, starts at 4.0)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Running cost per trip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Charged when a van leaves the depot (Electric vans: free)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Example fee (8 blocks, early, rating 4)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Base × rating × early tip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery staff and tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bought any time with credits from the Vans tab.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Group</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 1 (cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 2 (cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Level 3 (cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Total (cr)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery drivers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Staff</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Fleet of 3 vans, then 4, 5 and 6</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Driver training</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Vans drive 12% faster per level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Dispatcher</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Most urgent job goes first; promises 5 min longer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Handheld scanners</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tools</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Drop-offs take half the time; +1 cr tip each</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Route planner</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Delivery fees +15% per level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Bigger vans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each van carries 2 deliveries per trip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Electric vans</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Trips cost nothing to run</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Everything bought</t>
   </si>
 </sst>
 </file>
@@ -2524,4 +2649,345 @@
     <oddFooter/>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C11"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="72"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="14"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>216</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>180</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>217</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="C5" s="12" t="n">
+        <f aca="false">25+3*8</f>
+        <v>49</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>220</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="C6" s="12" t="n">
+        <f aca="false">2+0.25*8</f>
+        <v>4</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="C7" s="12" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>225</v>
+      </c>
+      <c r="C8" s="12" t="n">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>226</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>227</v>
+      </c>
+      <c r="C9" s="12" t="n">
+        <f aca="false">0.8+0.1*4</f>
+        <v>1.2</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>228</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>229</v>
+      </c>
+      <c r="C10" s="12" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>230</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>231</v>
+      </c>
+      <c r="C11" s="12" t="n">
+        <f aca="false">ROUND(C6*C9*C7,0)</f>
+        <v>6</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="20"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="9"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="48"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="4" style="0" width="12"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>232</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>233</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>165</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>234</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>150</v>
+      </c>
+      <c r="D4" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="E4" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="F4" s="11" t="s">
+        <v>237</v>
+      </c>
+      <c r="G4" s="11" t="s">
+        <v>238</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>239</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="C5" s="12" t="s">
+        <v>241</v>
+      </c>
+      <c r="D5" s="13" t="n">
+        <v>90</v>
+      </c>
+      <c r="E5" s="13" t="n">
+        <v>180</v>
+      </c>
+      <c r="F5" s="13" t="n">
+        <v>320</v>
+      </c>
+      <c r="G5" s="12" t="n">
+        <f aca="false">SUM(D5:F5)</f>
+        <v>590</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="C6" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="D6" s="13" t="n">
+        <v>70</v>
+      </c>
+      <c r="E6" s="13" t="n">
+        <v>150</v>
+      </c>
+      <c r="F6" s="13"/>
+      <c r="G6" s="12" t="n">
+        <f aca="false">SUM(D6:F6)</f>
+        <v>220</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>244</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>240</v>
+      </c>
+      <c r="C7" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="D7" s="13" t="n">
+        <v>110</v>
+      </c>
+      <c r="E7" s="13"/>
+      <c r="F7" s="13"/>
+      <c r="G7" s="12" t="n">
+        <f aca="false">SUM(D7:F7)</f>
+        <v>110</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C8" s="12" t="s">
+        <v>248</v>
+      </c>
+      <c r="D8" s="13" t="n">
+        <v>60</v>
+      </c>
+      <c r="E8" s="13"/>
+      <c r="F8" s="13"/>
+      <c r="G8" s="12" t="n">
+        <f aca="false">SUM(D8:F8)</f>
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>249</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C9" s="12" t="s">
+        <v>250</v>
+      </c>
+      <c r="D9" s="13" t="n">
+        <v>100</v>
+      </c>
+      <c r="E9" s="13" t="n">
+        <v>200</v>
+      </c>
+      <c r="F9" s="13"/>
+      <c r="G9" s="12" t="n">
+        <f aca="false">SUM(D9:F9)</f>
+        <v>300</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>251</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C10" s="12" t="s">
+        <v>252</v>
+      </c>
+      <c r="D10" s="13" t="n">
+        <v>160</v>
+      </c>
+      <c r="E10" s="13"/>
+      <c r="F10" s="13"/>
+      <c r="G10" s="12" t="n">
+        <f aca="false">SUM(D10:F10)</f>
+        <v>160</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>253</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>247</v>
+      </c>
+      <c r="C11" s="12" t="s">
+        <v>254</v>
+      </c>
+      <c r="D11" s="13" t="n">
+        <v>120</v>
+      </c>
+      <c r="E11" s="13"/>
+      <c r="F11" s="13"/>
+      <c r="G11" s="12" t="n">
+        <f aca="false">SUM(D11:F11)</f>
+        <v>120</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="7" t="s">
+        <v>255</v>
+      </c>
+      <c r="G13" s="7" t="n">
+        <f aca="false">SUM(G5:G11)</f>
+        <v>1560</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Ease delivery promises for the starting fleet
Promises get 5 more minutes and a late drop pulls the rating down less,
so a new player with three vans makes most drops on time.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014B4MfCeMGRMcDjRmBPkjgy
</commit_message>
<xml_diff>
--- a/WareTrack_game_rules.xlsx
+++ b/WareTrack_game_rules.xlsx
@@ -709,7 +709,7 @@
     <t xml:space="preserve">Promised time</t>
   </si>
   <si>
-    <t xml:space="preserve">Minutes from shipping until the drop is due: 25 + 3 per block of route (+5 with a Dispatcher)</t>
+    <t xml:space="preserve">Minutes from shipping until the drop is due: 30 + 3 per block of route (+5 with a Dispatcher)</t>
   </si>
   <si>
     <t xml:space="preserve">Base fee (credits)</t>
@@ -2693,8 +2693,8 @@
         <v>219</v>
       </c>
       <c r="C5" s="12" t="n">
-        <f aca="false">25+3*8</f>
-        <v>49</v>
+        <f aca="false">30+3*8</f>
+        <v>54</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">

</xml_diff>

<commit_message>
Connect the warehouses, deliver to every shop and home, tidy traffic
Transfer trucks now drive stock between warehouses on the public roads;
the Stock tab can request one, and other sites send them on their own.
Each site's neighbourhood gets ten houses, and orders go to every shop
and home. Shipment tracking gains an Outbound view that follows an order
from the pick queue to the door; shops and homes can be selected to see
their open orders and history.

Traffic: vehicles enter and leave on long approach roads instead of
appearing or vanishing on screen, cars no longer teleport at the map
edge, yard lanes allow one truck movement at a time so docking and
departing trucks never clip, and queued trucks never reverse. Fixes
broken licence plates on some trucks.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014B4MfCeMGRMcDjRmBPkjgy
</commit_message>
<xml_diff>
--- a/WareTrack_game_rules.xlsx
+++ b/WareTrack_game_rules.xlsx
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="277" uniqueCount="256">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="271">
   <si>
     <t xml:space="preserve">Shift calculator</t>
   </si>
@@ -697,6 +697,36 @@
     <t xml:space="preserve">Zooms out to all five sites with a name pin over each</t>
   </si>
   <si>
+    <t xml:space="preserve">Transfer trucks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">WareTrack trucks drive stock between your warehouses on the public roads, obeying the same lights and lanes</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every 90–160 min per site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Request a transfer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Stock tab: a nearby warehouse sends 5 pallets (4 of the product you need). Slower than Expedite but cheaper</t>
+  </si>
+  <si>
+    <t xml:space="preserve">15 points</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Yard lane</t>
+  </si>
+  <si>
+    <t xml:space="preserve">One truck moves in a yard lane at a time: a truck only backs into a dock or pulls out when the lane is clear</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Approach roads</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Traffic enters and leaves the map along long approach roads, so vehicles never pop in or vanish on screen</t>
+  </si>
+  <si>
     <t xml:space="preserve">Delivery vans</t>
   </si>
   <si>
@@ -746,6 +776,21 @@
   </si>
   <si>
     <t xml:space="preserve">Base × rating × early tip</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Customers</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every shop and every house in the city around the site you run: 8 shops and 10 homes per site, plus shops you build</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 per site</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Tracking</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Shipment tracking → Outbound follows an order: placed, picked, staged, shipped, out for delivery, delivered. Tap a shop or house to see its open orders</t>
   </si>
   <si>
     <t xml:space="preserve">Delivery staff and tools</t>
@@ -2477,7 +2522,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="26"/>
@@ -2637,6 +2682,50 @@
         <v>214</v>
       </c>
       <c r="C16" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>215</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>216</v>
+      </c>
+      <c r="C17" s="12" t="s">
+        <v>217</v>
+      </c>
+    </row>
+    <row r="18" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="12" t="s">
+        <v>218</v>
+      </c>
+      <c r="B18" s="12" t="s">
+        <v>219</v>
+      </c>
+      <c r="C18" s="12" t="s">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="19" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="12" t="s">
+        <v>221</v>
+      </c>
+      <c r="B19" s="12" t="s">
+        <v>222</v>
+      </c>
+      <c r="C19" s="12" t="s">
+        <v>212</v>
+      </c>
+    </row>
+    <row r="20" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="12" t="s">
+        <v>223</v>
+      </c>
+      <c r="B20" s="12" t="s">
+        <v>224</v>
+      </c>
+      <c r="C20" s="12" t="s">
         <v>212</v>
       </c>
     </row>
@@ -2656,7 +2745,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:C11"/>
+  <dimension ref="A1:C13"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="34"/>
@@ -2666,12 +2755,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>215</v>
+        <v>225</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>216</v>
+        <v>226</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2679,7 +2768,7 @@
         <v>180</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>217</v>
+        <v>227</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>181</v>
@@ -2687,10 +2776,10 @@
     </row>
     <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>218</v>
+        <v>228</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>219</v>
+        <v>229</v>
       </c>
       <c r="C5" s="12" t="n">
         <f aca="false">30+3*8</f>
@@ -2699,10 +2788,10 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>220</v>
+        <v>230</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>221</v>
+        <v>231</v>
       </c>
       <c r="C6" s="12" t="n">
         <f aca="false">2+0.25*8</f>
@@ -2711,10 +2800,10 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>222</v>
+        <v>232</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>223</v>
+        <v>233</v>
       </c>
       <c r="C7" s="12" t="n">
         <v>1.25</v>
@@ -2722,10 +2811,10 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>224</v>
+        <v>234</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>225</v>
+        <v>235</v>
       </c>
       <c r="C8" s="12" t="n">
         <v>0.5</v>
@@ -2733,10 +2822,10 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>226</v>
+        <v>236</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>227</v>
+        <v>237</v>
       </c>
       <c r="C9" s="12" t="n">
         <f aca="false">0.8+0.1*4</f>
@@ -2745,10 +2834,10 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>228</v>
+        <v>238</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>229</v>
+        <v>239</v>
       </c>
       <c r="C10" s="12" t="n">
         <v>2</v>
@@ -2756,14 +2845,36 @@
     </row>
     <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>230</v>
+        <v>240</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>231</v>
+        <v>241</v>
       </c>
       <c r="C11" s="12" t="n">
         <f aca="false">ROUND(C6*C9*C7,0)</f>
         <v>6</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
+        <v>242</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>243</v>
+      </c>
+      <c r="C12" s="12" t="s">
+        <v>244</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
+        <v>245</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>246</v>
+      </c>
+      <c r="C13" s="12" t="s">
+        <v>212</v>
       </c>
     </row>
   </sheetData>
@@ -2793,12 +2904,12 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>247</v>
       </c>
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="2" t="s">
-        <v>233</v>
+        <v>248</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2806,33 +2917,33 @@
         <v>165</v>
       </c>
       <c r="B4" s="11" t="s">
-        <v>234</v>
+        <v>249</v>
       </c>
       <c r="C4" s="11" t="s">
         <v>150</v>
       </c>
       <c r="D4" s="11" t="s">
-        <v>235</v>
+        <v>250</v>
       </c>
       <c r="E4" s="11" t="s">
-        <v>236</v>
+        <v>251</v>
       </c>
       <c r="F4" s="11" t="s">
-        <v>237</v>
+        <v>252</v>
       </c>
       <c r="G4" s="11" t="s">
-        <v>238</v>
+        <v>253</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="12" t="s">
-        <v>239</v>
+        <v>254</v>
       </c>
       <c r="B5" s="12" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="C5" s="12" t="s">
-        <v>241</v>
+        <v>256</v>
       </c>
       <c r="D5" s="13" t="n">
         <v>90</v>
@@ -2850,13 +2961,13 @@
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="12" t="s">
-        <v>242</v>
+        <v>257</v>
       </c>
       <c r="B6" s="12" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="C6" s="12" t="s">
-        <v>243</v>
+        <v>258</v>
       </c>
       <c r="D6" s="13" t="n">
         <v>70</v>
@@ -2872,13 +2983,13 @@
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="12" t="s">
-        <v>244</v>
+        <v>259</v>
       </c>
       <c r="B7" s="12" t="s">
-        <v>240</v>
+        <v>255</v>
       </c>
       <c r="C7" s="12" t="s">
-        <v>245</v>
+        <v>260</v>
       </c>
       <c r="D7" s="13" t="n">
         <v>110</v>
@@ -2892,13 +3003,13 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="12" t="s">
-        <v>246</v>
+        <v>261</v>
       </c>
       <c r="B8" s="12" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C8" s="12" t="s">
-        <v>248</v>
+        <v>263</v>
       </c>
       <c r="D8" s="13" t="n">
         <v>60</v>
@@ -2912,13 +3023,13 @@
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="12" t="s">
-        <v>249</v>
+        <v>264</v>
       </c>
       <c r="B9" s="12" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C9" s="12" t="s">
-        <v>250</v>
+        <v>265</v>
       </c>
       <c r="D9" s="13" t="n">
         <v>100</v>
@@ -2934,13 +3045,13 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="12" t="s">
-        <v>251</v>
+        <v>266</v>
       </c>
       <c r="B10" s="12" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C10" s="12" t="s">
-        <v>252</v>
+        <v>267</v>
       </c>
       <c r="D10" s="13" t="n">
         <v>160</v>
@@ -2954,13 +3065,13 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="12" t="s">
-        <v>253</v>
+        <v>268</v>
       </c>
       <c r="B11" s="12" t="s">
-        <v>247</v>
+        <v>262</v>
       </c>
       <c r="C11" s="12" t="s">
-        <v>254</v>
+        <v>269</v>
       </c>
       <c r="D11" s="13" t="n">
         <v>120</v>
@@ -2974,7 +3085,7 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="7" t="s">
-        <v>255</v>
+        <v>270</v>
       </c>
       <c r="G13" s="7" t="n">
         <f aca="false">SUM(G5:G11)</f>

</xml_diff>

<commit_message>
Add order requests, Hands-on mode, missions and a bigger world
During shifts every new order pops up in an Actions card with a timer;
accept, rush or decline it, or lose the customer. Hands-on mode makes
you dock every truck, release every order and send every van yourself
for 1.25x points. Three rotating missions pay credits and XP with a
chest every fifth one, on-time deliveries build a streak that raises
fees, and the game pays out what your network earned while you were
away. The town gains North and South districts with new streets and
homes that open with the fifth van, and a new three-mood soundtrack.

Fixes a crash when hovering city houses in Town mode, oversized icons
in the shift report, and the missing favicon.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014B4MfCeMGRMcDjRmBPkjgy
</commit_message>
<xml_diff>
--- a/WareTrack_game_rules.xlsx
+++ b/WareTrack_game_rules.xlsx
@@ -17,6 +17,7 @@
     <sheet name="World and traffic" sheetId="7" state="visible" r:id="rId9"/>
     <sheet name="Deliveries" sheetId="8" state="visible" r:id="rId10"/>
     <sheet name="Delivery upgrades" sheetId="9" state="visible" r:id="rId11"/>
+    <sheet name="Challenge and rewards" sheetId="10" state="visible" r:id="rId12"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -50,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="295" uniqueCount="271">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="331" uniqueCount="305">
   <si>
     <t xml:space="preserve">Shift calculator</t>
   </si>
@@ -863,6 +864,108 @@
   </si>
   <si>
     <t xml:space="preserve">Everything bought</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order requests, Hands-on mode, missions and streaks</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The systems that give each session a goal and a reason to come back.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">System</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Order request window</t>
+  </si>
+  <si>
+    <t xml:space="preserve">During a shift every new order pops up in the Actions card. Accept, rush it or decline before the timer runs out (real seconds, paused when the game is paused)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missed request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">The customer goes elsewhere: points lost and customer rating drops</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating cost of a missed request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Applied to the 0–5 customer rating</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rating cost of declining</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Declining is cheaper than ignoring</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Rush an order</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accept as rush: due in 25 minutes, pays the rush bonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Out-of-stock request</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Accepting sends a transfer truck from another warehouse automatically (15 points)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hands-on mode</t>
+  </si>
+  <si>
+    <t xml:space="preserve">You dock every truck, release every order to the floor and send every van yourself; all points earned are multiplied</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Missions</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3 active missions from 11 types (put-aways, on-time orders, deliveries, home drops, early drops, delivery credits, fast trucks, streaks, combos, transfers, 2-star shifts); targets and rewards grow with level</t>
+  </si>
+  <si>
+    <t xml:space="preserve">30–60 cr + XP</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Mission chest</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Every 5th mission completed</t>
+  </si>
+  <si>
+    <t xml:space="preserve">On-time delivery streak</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Each consecutive on-time drop adds to every delivery fee; a late drop resets it</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+2.5% per drop</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Streak cap</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Highest streak bonus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">+25%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Welcome-back pay</t>
+  </si>
+  <si>
+    <t xml:space="preserve">While you are away your network keeps earning; counted for up to 8 hours</t>
+  </si>
+  <si>
+    <t xml:space="preserve">14 cr/h + upgrades</t>
+  </si>
+  <si>
+    <t xml:space="preserve">North and South districts</t>
+  </si>
+  <si>
+    <t xml:space="preserve">18 more homes per site, further out and better paid; open with the first Delivery drivers upgrade</t>
+  </si>
+  <si>
+    <t xml:space="preserve">5th van</t>
   </si>
 </sst>
 </file>
@@ -1552,6 +1655,194 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="30"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="92"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>271</v>
+      </c>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="2" t="s">
+        <v>272</v>
+      </c>
+    </row>
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A4" s="11" t="s">
+        <v>273</v>
+      </c>
+      <c r="B4" s="11" t="s">
+        <v>227</v>
+      </c>
+      <c r="C4" s="11" t="s">
+        <v>181</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="12" t="s">
+        <v>274</v>
+      </c>
+      <c r="B5" s="12" t="s">
+        <v>275</v>
+      </c>
+      <c r="C5" s="13" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="12" t="s">
+        <v>276</v>
+      </c>
+      <c r="B6" s="12" t="s">
+        <v>277</v>
+      </c>
+      <c r="C6" s="13" t="n">
+        <v>-5</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="12" t="s">
+        <v>278</v>
+      </c>
+      <c r="B7" s="12" t="s">
+        <v>279</v>
+      </c>
+      <c r="C7" s="13" t="n">
+        <v>-0.15</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="12" t="s">
+        <v>280</v>
+      </c>
+      <c r="B8" s="12" t="s">
+        <v>281</v>
+      </c>
+      <c r="C8" s="13" t="n">
+        <v>-0.05</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="12" t="s">
+        <v>282</v>
+      </c>
+      <c r="B9" s="12" t="s">
+        <v>283</v>
+      </c>
+      <c r="C9" s="13" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="12" t="s">
+        <v>284</v>
+      </c>
+      <c r="B10" s="12" t="s">
+        <v>285</v>
+      </c>
+      <c r="C10" s="13" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" customFormat="false" ht="26.85" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="12" t="s">
+        <v>286</v>
+      </c>
+      <c r="B11" s="12" t="s">
+        <v>287</v>
+      </c>
+      <c r="C11" s="13" t="n">
+        <v>1.25</v>
+      </c>
+    </row>
+    <row r="12" customFormat="false" ht="39.55" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="12" t="s">
+        <v>288</v>
+      </c>
+      <c r="B12" s="12" t="s">
+        <v>289</v>
+      </c>
+      <c r="C12" s="13" t="s">
+        <v>290</v>
+      </c>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="12" t="s">
+        <v>291</v>
+      </c>
+      <c r="B13" s="12" t="s">
+        <v>292</v>
+      </c>
+      <c r="C13" s="13" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="12" t="s">
+        <v>293</v>
+      </c>
+      <c r="B14" s="12" t="s">
+        <v>294</v>
+      </c>
+      <c r="C14" s="13" t="s">
+        <v>295</v>
+      </c>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="12" t="s">
+        <v>296</v>
+      </c>
+      <c r="B15" s="12" t="s">
+        <v>297</v>
+      </c>
+      <c r="C15" s="13" t="s">
+        <v>298</v>
+      </c>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="12" t="s">
+        <v>299</v>
+      </c>
+      <c r="B16" s="12" t="s">
+        <v>300</v>
+      </c>
+      <c r="C16" s="13" t="s">
+        <v>301</v>
+      </c>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="12" t="s">
+        <v>302</v>
+      </c>
+      <c r="B17" s="12" t="s">
+        <v>303</v>
+      </c>
+      <c r="C17" s="13" t="s">
+        <v>304</v>
+      </c>
+    </row>
+  </sheetData>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <sheetPr filterMode="false">

</xml_diff>